<commit_message>
create collect gap evidence
</commit_message>
<xml_diff>
--- a/Scorecards.xlsx
+++ b/Scorecards.xlsx
@@ -8,13 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\sql\ssas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF94C113-70B0-4384-8130-02AA52CD4CEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F092FB7F-F66F-4CDB-8381-0CE81F89FF0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{7CE94D96-0740-4CB8-A656-FD85CCF7F4E0}"/>
   </bookViews>
   <sheets>
     <sheet name="Scorecard" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Scorecard!$A$1:$AD$55</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -327,12 +330,24 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -347,9 +362,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -669,8 +686,8 @@
   <cols>
     <col min="1" max="1" width="3.5703125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="79.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.140625" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="18" hidden="1" customWidth="1"/>
     <col min="5" max="5" width="11.140625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="13.28515625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="14.28515625" bestFit="1" customWidth="1"/>
@@ -688,8 +705,8 @@
     <col min="19" max="19" width="18.28515625" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="16.140625" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="14.85546875" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="14.7109375" customWidth="1"/>
+    <col min="23" max="23" width="12.42578125" customWidth="1"/>
     <col min="24" max="24" width="16.140625" bestFit="1" customWidth="1"/>
     <col min="25" max="25" width="12.5703125" bestFit="1" customWidth="1"/>
     <col min="26" max="26" width="13.7109375" bestFit="1" customWidth="1"/>
@@ -745,49 +762,49 @@
       <c r="O1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="X1" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Y1" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="Z1" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AA1" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="AB1" s="1" t="s">
+      <c r="AB1" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="AC1" s="1" t="s">
+      <c r="AC1" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="AD1" s="1" t="s">
+      <c r="AD1" s="2" t="s">
         <v>28</v>
       </c>
     </row>
@@ -5568,6 +5585,11 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:AD55" xr:uid="{93B65446-B849-42AD-A0BF-0F2E9FDAA696}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:AD55">
+      <sortCondition descending="1" ref="V1:V55"/>
+    </sortState>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>